<commit_message>
Update reports 2026-10-13 10:07
</commit_message>
<xml_diff>
--- a/gex_pivot_levels_2026-10-13.xlsx
+++ b/gex_pivot_levels_2026-10-13.xlsx
@@ -15,12 +15,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Pivots" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ES'!$A$1:$G$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ES'!$A$1:$G$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'NQ'!$A$1:$G$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RTY'!$A$1:$G$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CL'!$A$1:$G$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'GC'!$A$1:$G$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All Pivots'!$A$1:$H$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All Pivots'!$A$1:$H$66</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -544,12 +544,12 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>-$7.99M</t>
+          <t>-$7.04M</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>+$8.39M</t>
+          <t>+$7.38M</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -573,12 +573,12 @@
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>-$10.93M</t>
+          <t>-$9.66M</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>+$15.07M</t>
+          <t>+$13.32M</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -606,12 +606,12 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>-$9.49M</t>
+          <t>-$8.47M</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>+$17.66M</t>
+          <t>+$15.77M</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -668,12 +668,12 @@
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>+$1.59M</t>
+          <t>+$1.45M</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>+$32.51M</t>
+          <t>+$29.80M</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
@@ -734,12 +734,12 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>-$12.52M</t>
+          <t>-$12.28M</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>+$23.48M</t>
+          <t>+$23.03M</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -767,12 +767,12 @@
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>+$18.62M</t>
+          <t>+$18.94M</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>+$51.12M</t>
+          <t>+$52.01M</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -796,12 +796,12 @@
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>+$22.68M</t>
+          <t>+$23.45M</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>+$49.07M</t>
+          <t>+$50.73M</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -862,12 +862,12 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>-$6.77M</t>
+          <t>-$7.17M</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>+$34.14M</t>
+          <t>+$36.18M</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -895,12 +895,12 @@
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>+$18.21M</t>
+          <t>+$19.49M</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>+$28.00M</t>
+          <t>+$29.97M</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -928,12 +928,12 @@
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>+$6.41M</t>
+          <t>+$7.01M</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>+$17.90M</t>
+          <t>+$19.58M</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -961,12 +961,12 @@
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>+$34.82M</t>
+          <t>+$38.73M</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>+$44.15M</t>
+          <t>+$49.11M</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
@@ -1015,43 +1015,39 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>7883.88</v>
+        <v>7872.51</v>
       </c>
       <c r="B17" s="2" t="n">
-        <v>782</v>
+        <v>7835</v>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>+$2.62M</t>
+          <t>+$11.58M</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>+$19.18M</t>
+          <t>+$15.48M</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>7887.51</v>
+        <v>7882.51</v>
       </c>
       <c r="B18" s="2" t="n">
-        <v>7850</v>
+        <v>7845</v>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
@@ -1060,56 +1056,126 @@
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>+$10.95M</t>
+          <t>+$4.49M</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>+$16.50M</t>
+          <t>+$6.97M</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
+        <v>7883.88</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>782</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>+$2.62M</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>+$19.18M</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="n">
+        <v>7887.51</v>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>7850</v>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>+$12.55M</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>+$18.92M</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
         <v>7903.95</v>
       </c>
-      <c r="B19" s="2" t="n">
+      <c r="B21" s="2" t="n">
         <v>784</v>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="D19" s="9" t="inlineStr">
+      <c r="D21" s="9" t="inlineStr">
         <is>
           <t>+$10.90M</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="E21" s="3" t="inlineStr">
         <is>
           <t>+$11.37M</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G19"/>
+  <autoFilter ref="A1:G21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2794,7 +2860,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H64"/>
+  <dimension ref="A1:H66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2932,36 +2998,32 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>7823.68</v>
+        <v>7837.51</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>776</v>
+        <v>7800</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>+$9.84M</t>
+          <t>+$18.94M</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>+$51.63M</t>
+          <t>+$52.01M</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -2970,32 +3032,36 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>7837.51</v>
+        <v>7823.68</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>7800</v>
+        <v>776</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>+$18.62M</t>
+          <t>+$9.84M</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>+$51.12M</t>
+          <t>+$51.63M</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -3016,12 +3082,12 @@
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>+$22.68M</t>
+          <t>+$23.45M</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>+$49.07M</t>
+          <t>+$50.73M</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -3042,24 +3108,24 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>7863.81</v>
+        <v>7862.51</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>780</v>
+        <v>7825</v>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>+$8.86M</t>
+          <t>+$38.73M</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>+$46.40M</t>
+          <t>+$49.11M</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
@@ -3080,24 +3146,24 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>7862.51</v>
+        <v>7863.81</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>7825</v>
+        <v>780</v>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>+$34.82M</t>
+          <t>+$8.86M</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>+$44.15M</t>
+          <t>+$46.40M</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
@@ -3168,12 +3234,12 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>-$6.77M</t>
+          <t>-$7.17M</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>+$34.14M</t>
+          <t>+$36.18M</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
@@ -3188,40 +3254,40 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B11" s="5" t="n">
-        <v>7807.51</v>
-      </c>
-      <c r="C11" s="5" t="n">
-        <v>7770</v>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E11" s="8" t="inlineStr">
-        <is>
-          <t>+$1.59M</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>+$32.51M</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
+      <c r="B11" s="2" t="n">
+        <v>7803.61</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>774</v>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>-$7.66M</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>+$30.23M</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -3232,24 +3298,24 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>7803.61</v>
+        <v>7852.51</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>774</v>
+        <v>7815</v>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>-$7.66M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>+$19.49M</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>+$30.23M</t>
+          <t>+$29.97M</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -3259,43 +3325,43 @@
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
-        <v>7852.51</v>
-      </c>
-      <c r="C13" s="2" t="n">
-        <v>7815</v>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="B13" s="5" t="n">
+        <v>7807.51</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>7770</v>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E13" s="9" t="inlineStr">
-        <is>
-          <t>+$18.21M</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>+$28.00M</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>+$1.45M</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>+$29.80M</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -3320,12 +3386,12 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>-$12.52M</t>
+          <t>-$12.28M</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>+$23.48M</t>
+          <t>+$23.03M</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
@@ -3380,24 +3446,24 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>7883.88</v>
+        <v>7857.51</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>782</v>
+        <v>7820</v>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>+$2.62M</t>
+          <t>+$7.01M</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>+$19.18M</t>
+          <t>+$19.58M</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
@@ -3414,28 +3480,28 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>4304.81</v>
+        <v>7883.88</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>90.5</v>
+        <v>782</v>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>GDX</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>+$17.96M</t>
+          <t>+$2.62M</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>+$18.02M</t>
+          <t>+$19.18M</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -3445,81 +3511,85 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>7887.51</v>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>7850</v>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>+$12.55M</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>+$18.92M</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
           <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="n">
-        <v>7857.51</v>
-      </c>
-      <c r="C18" s="2" t="n">
-        <v>7820</v>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E18" s="9" t="inlineStr">
-        <is>
-          <t>+$6.41M</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>+$17.90M</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>7797.51</v>
+        <v>4304.81</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>7760</v>
+        <v>90.5</v>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>-$9.49M</t>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>+$17.96M</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>+$17.66M</t>
+          <t>+$18.02M</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H19" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -3528,24 +3598,24 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>7887.51</v>
+        <v>7797.51</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>7850</v>
+        <v>7760</v>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E20" s="9" t="inlineStr">
-        <is>
-          <t>+$10.95M</t>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>-$8.47M</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>+$16.50M</t>
+          <t>+$15.77M</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
@@ -3556,114 +3626,110 @@
       <c r="H20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B21" s="5" t="n">
-        <v>7787.51</v>
-      </c>
-      <c r="C21" s="5" t="n">
-        <v>7750</v>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="B21" s="2" t="n">
+        <v>7872.51</v>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>7835</v>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr">
-        <is>
-          <t>-$10.93M</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="inlineStr">
-        <is>
-          <t>+$15.07M</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H21" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>+$11.58M</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>+$15.48M</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>7787.51</v>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>7750</v>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>-$9.66M</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>+$13.32M</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
           <t>RTY</t>
         </is>
       </c>
-      <c r="B22" s="5" t="n">
+      <c r="B23" s="5" t="n">
         <v>2826.86</v>
       </c>
-      <c r="C22" s="5" t="n">
+      <c r="C23" s="5" t="n">
         <v>281</v>
       </c>
-      <c r="D22" s="6" t="inlineStr">
+      <c r="D23" s="6" t="inlineStr">
         <is>
           <t>IWM</t>
         </is>
       </c>
-      <c r="E22" s="8" t="inlineStr">
+      <c r="E23" s="8" t="inlineStr">
         <is>
           <t>+$6.17M</t>
         </is>
       </c>
-      <c r="F22" s="6" t="inlineStr">
+      <c r="F23" s="6" t="inlineStr">
         <is>
           <t>+$12.68M</t>
         </is>
       </c>
-      <c r="G22" s="6" t="inlineStr">
+      <c r="G23" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H22" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="n">
-        <v>7903.95</v>
-      </c>
-      <c r="C23" s="2" t="n">
-        <v>784</v>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E23" s="9" t="inlineStr">
-        <is>
-          <t>+$10.90M</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>+$11.37M</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr">
+      <c r="H23" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -3672,74 +3738,74 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>7903.95</v>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>784</v>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>+$10.90M</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>+$11.37M</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B24" s="2" t="n">
+      <c r="B25" s="2" t="n">
         <v>30711.96</v>
       </c>
-      <c r="C24" s="2" t="n">
+      <c r="C25" s="2" t="n">
         <v>747</v>
       </c>
-      <c r="D24" s="3" t="inlineStr">
+      <c r="D25" s="3" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>-$1.57M</t>
         </is>
       </c>
-      <c r="F24" s="3" t="inlineStr">
+      <c r="F25" s="3" t="inlineStr">
         <is>
           <t>+$11.29M</t>
         </is>
       </c>
-      <c r="G24" s="3" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H24" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="n">
-        <v>4209.67</v>
-      </c>
-      <c r="C25" s="5" t="n">
-        <v>88.5</v>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E25" s="8" t="inlineStr">
-        <is>
-          <t>+$10.03M</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
-          <t>+$10.99M</t>
-        </is>
-      </c>
-      <c r="G25" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H25" s="6" t="inlineStr">
+      <c r="H25" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -3752,10 +3818,10 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>4447.51</v>
+        <v>4209.67</v>
       </c>
       <c r="C26" s="5" t="n">
-        <v>93.5</v>
+        <v>88.5</v>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
@@ -3764,12 +3830,12 @@
       </c>
       <c r="E26" s="8" t="inlineStr">
         <is>
-          <t>+$9.35M</t>
+          <t>+$10.03M</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>+$9.43M</t>
+          <t>+$10.99M</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
@@ -3790,70 +3856,74 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
+        <v>4447.51</v>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>93.5</v>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>+$9.35M</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>+$9.43M</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
         <v>4187.41</v>
       </c>
-      <c r="C27" s="5" t="n">
+      <c r="C28" s="5" t="n">
         <v>380</v>
       </c>
-      <c r="D27" s="6" t="inlineStr">
+      <c r="D28" s="6" t="inlineStr">
         <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="E27" s="8" t="inlineStr">
+      <c r="E28" s="8" t="inlineStr">
         <is>
           <t>+$6.95M</t>
         </is>
       </c>
-      <c r="F27" s="6" t="inlineStr">
+      <c r="F28" s="6" t="inlineStr">
         <is>
           <t>+$8.53M</t>
         </is>
       </c>
-      <c r="G27" s="6" t="inlineStr">
+      <c r="G28" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H27" s="6" t="inlineStr">
+      <c r="H28" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="n">
-        <v>7767.51</v>
-      </c>
-      <c r="C28" s="2" t="n">
-        <v>7730</v>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t>-$7.99M</t>
-        </is>
-      </c>
-      <c r="F28" s="3" t="inlineStr">
-        <is>
-          <t>+$8.39M</t>
-        </is>
-      </c>
-      <c r="G28" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
@@ -3972,28 +4042,28 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>4518.86</v>
+        <v>7767.51</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>95</v>
+        <v>7730</v>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E32" s="9" t="inlineStr">
-        <is>
-          <t>+$1.58M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>-$7.04M</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>+$4.73M</t>
+          <t>+$7.38M</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
@@ -4006,78 +4076,74 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>7882.51</v>
+      </c>
+      <c r="C33" s="2" t="n">
+        <v>7845</v>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E33" s="9" t="inlineStr">
+        <is>
+          <t>+$4.49M</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>+$6.97M</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B33" s="2" t="n">
-        <v>4376.16</v>
-      </c>
-      <c r="C33" s="2" t="n">
-        <v>92</v>
-      </c>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="B34" s="2" t="n">
+        <v>4518.86</v>
+      </c>
+      <c r="C34" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>-$1.47M</t>
-        </is>
-      </c>
-      <c r="F33" s="3" t="inlineStr">
-        <is>
-          <t>+$4.59M</t>
-        </is>
-      </c>
-      <c r="G33" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H33" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="6" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B34" s="5" t="n">
-        <v>92.01000000000001</v>
-      </c>
-      <c r="C34" s="5" t="n">
-        <v>150</v>
-      </c>
-      <c r="D34" s="6" t="inlineStr">
-        <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E34" s="8" t="inlineStr">
-        <is>
-          <t>+$846.88K</t>
-        </is>
-      </c>
-      <c r="F34" s="6" t="inlineStr">
-        <is>
-          <t>+$2.07M</t>
-        </is>
-      </c>
-      <c r="G34" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H34" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="E34" s="9" t="inlineStr">
+        <is>
+          <t>+$1.58M</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>+$4.73M</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -4086,206 +4152,210 @@
         </is>
       </c>
       <c r="B35" s="2" t="n">
+        <v>4376.16</v>
+      </c>
+      <c r="C35" s="2" t="n">
+        <v>92</v>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>-$1.47M</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>+$4.59M</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>92.01000000000001</v>
+      </c>
+      <c r="C36" s="5" t="n">
+        <v>150</v>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>+$846.88K</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>+$2.07M</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="n">
         <v>4220.47</v>
       </c>
-      <c r="C35" s="2" t="n">
+      <c r="C37" s="2" t="n">
         <v>383</v>
       </c>
-      <c r="D35" s="3" t="inlineStr">
+      <c r="D37" s="3" t="inlineStr">
         <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="E35" s="9" t="inlineStr">
+      <c r="E37" s="9" t="inlineStr">
         <is>
           <t>+$522.50K</t>
         </is>
       </c>
-      <c r="F35" s="3" t="inlineStr">
+      <c r="F37" s="3" t="inlineStr">
         <is>
           <t>+$2.01M</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="G37" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H35" s="3" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="3" t="inlineStr">
+      <c r="H37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
         <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B36" s="2" t="n">
+      <c r="B38" s="2" t="n">
         <v>4328.59</v>
       </c>
-      <c r="C36" s="2" t="n">
+      <c r="C38" s="2" t="n">
         <v>91</v>
       </c>
-      <c r="D36" s="3" t="inlineStr">
+      <c r="D38" s="3" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="E36" s="4" t="inlineStr">
+      <c r="E38" s="4" t="inlineStr">
         <is>
           <t>-$44.35K</t>
         </is>
       </c>
-      <c r="F36" s="3" t="inlineStr">
+      <c r="F38" s="3" t="inlineStr">
         <is>
           <t>+$1.85M</t>
         </is>
       </c>
-      <c r="G36" s="3" t="inlineStr">
+      <c r="G38" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H36" s="3" t="inlineStr">
+      <c r="H38" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="6" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
         <is>
           <t>CL</t>
         </is>
       </c>
-      <c r="B37" s="5" t="n">
+      <c r="B39" s="5" t="n">
         <v>95.08</v>
       </c>
-      <c r="C37" s="5" t="n">
+      <c r="C39" s="5" t="n">
         <v>155</v>
       </c>
-      <c r="D37" s="6" t="inlineStr">
+      <c r="D39" s="6" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="E37" s="8" t="inlineStr">
+      <c r="E39" s="8" t="inlineStr">
         <is>
           <t>+$886.35K</t>
         </is>
       </c>
-      <c r="F37" s="6" t="inlineStr">
+      <c r="F39" s="6" t="inlineStr">
         <is>
           <t>+$1.10M</t>
         </is>
       </c>
-      <c r="G37" s="6" t="inlineStr">
+      <c r="G39" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H37" s="6" t="inlineStr">
+      <c r="H39" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="6" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B38" s="5" t="n">
-        <v>90.78</v>
-      </c>
-      <c r="C38" s="5" t="n">
-        <v>148</v>
-      </c>
-      <c r="D38" s="6" t="inlineStr">
-        <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E38" s="7" t="inlineStr">
-        <is>
-          <t>-$568.68K</t>
-        </is>
-      </c>
-      <c r="F38" s="6" t="inlineStr">
-        <is>
-          <t>+$1.01M</t>
-        </is>
-      </c>
-      <c r="G38" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H38" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="n">
-        <v>88.94</v>
-      </c>
-      <c r="C39" s="2" t="n">
-        <v>145</v>
-      </c>
-      <c r="D39" s="3" t="inlineStr">
-        <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E39" s="4" t="inlineStr">
-        <is>
-          <t>-$131.26K</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>+$628.13K</t>
-        </is>
-      </c>
-      <c r="G39" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>30807.8</v>
+        <v>90.78</v>
       </c>
       <c r="C40" s="5" t="n">
-        <v>30800</v>
+        <v>148</v>
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E40" s="8" t="inlineStr">
-        <is>
-          <t>+$358.16K</t>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>-$568.68K</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>+$574.04K</t>
+          <t>+$1.01M</t>
         </is>
       </c>
       <c r="G40" s="6" t="inlineStr">
@@ -4295,73 +4365,69 @@
       </c>
       <c r="H40" s="6" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>4257.24</v>
+        <v>88.94</v>
       </c>
       <c r="C41" s="2" t="n">
-        <v>89.5</v>
+        <v>145</v>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>GDX</t>
+          <t>USO</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>-$22.35K</t>
+          <t>-$131.26K</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>+$424.85K</t>
+          <t>+$628.13K</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H41" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>82.81</v>
+        <v>30807.8</v>
       </c>
       <c r="C42" s="5" t="n">
-        <v>135</v>
+        <v>30800</v>
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E42" s="7" t="inlineStr">
-        <is>
-          <t>-$384.67K</t>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>+$358.16K</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr">
         <is>
-          <t>+$397.70K</t>
+          <t>+$574.04K</t>
         </is>
       </c>
       <c r="G42" s="6" t="inlineStr">
@@ -4371,77 +4437,81 @@
       </c>
       <c r="H42" s="6" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>30707.8</v>
+        <v>4257.24</v>
       </c>
       <c r="C43" s="2" t="n">
-        <v>30700</v>
+        <v>89.5</v>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E43" s="9" t="inlineStr">
-        <is>
-          <t>+$49.68K</t>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>-$22.35K</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>+$369.82K</t>
+          <t>+$424.85K</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H43" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" s="3" t="inlineStr">
+      <c r="A44" s="6" t="inlineStr">
         <is>
           <t>CL</t>
         </is>
       </c>
-      <c r="B44" s="2" t="n">
-        <v>94.45999999999999</v>
-      </c>
-      <c r="C44" s="2" t="n">
-        <v>154</v>
-      </c>
-      <c r="D44" s="3" t="inlineStr">
+      <c r="B44" s="5" t="n">
+        <v>82.81</v>
+      </c>
+      <c r="C44" s="5" t="n">
+        <v>135</v>
+      </c>
+      <c r="D44" s="6" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="E44" s="9" t="inlineStr">
-        <is>
-          <t>+$250.80K</t>
-        </is>
-      </c>
-      <c r="F44" s="3" t="inlineStr">
-        <is>
-          <t>+$270.43K</t>
-        </is>
-      </c>
-      <c r="G44" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H44" s="3" t="inlineStr">
+      <c r="E44" s="7" t="inlineStr">
+        <is>
+          <t>-$384.67K</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="inlineStr">
+        <is>
+          <t>+$397.70K</t>
+        </is>
+      </c>
+      <c r="G44" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -4450,28 +4520,28 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>98.14</v>
+        <v>30707.8</v>
       </c>
       <c r="C45" s="2" t="n">
-        <v>160</v>
+        <v>30700</v>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>USO</t>
+          <t>NDX</t>
         </is>
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>+$254.47K</t>
+          <t>+$49.68K</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>+$263.76K</t>
+          <t>+$369.82K</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
@@ -4488,58 +4558,62 @@
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>85.87</v>
+        <v>94.45999999999999</v>
       </c>
       <c r="C46" s="2" t="n">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="E46" s="4" t="inlineStr">
-        <is>
-          <t>-$225.98K</t>
+      <c r="E46" s="9" t="inlineStr">
+        <is>
+          <t>+$250.80K</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>+$258.12K</t>
+          <t>+$270.43K</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H46" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>30727.8</v>
+        <v>98.14</v>
       </c>
       <c r="C47" s="2" t="n">
-        <v>30720</v>
+        <v>160</v>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E47" s="4" t="inlineStr">
-        <is>
-          <t>-$38.64K</t>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E47" s="9" t="inlineStr">
+        <is>
+          <t>+$254.47K</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>+$226.31K</t>
+          <t>+$263.76K</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
@@ -4552,78 +4626,70 @@
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="n">
+        <v>85.87</v>
+      </c>
+      <c r="C48" s="2" t="n">
+        <v>140</v>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>-$225.98K</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>+$258.12K</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B48" s="2" t="n">
-        <v>30697.8</v>
-      </c>
-      <c r="C48" s="2" t="n">
-        <v>30690</v>
-      </c>
-      <c r="D48" s="3" t="inlineStr">
+      <c r="B49" s="2" t="n">
+        <v>30727.8</v>
+      </c>
+      <c r="C49" s="2" t="n">
+        <v>30720</v>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E48" s="4" t="inlineStr">
-        <is>
-          <t>-$60.72K</t>
-        </is>
-      </c>
-      <c r="F48" s="3" t="inlineStr">
-        <is>
-          <t>+$215.27K</t>
-        </is>
-      </c>
-      <c r="G48" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H48" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B49" s="5" t="n">
-        <v>30657.8</v>
-      </c>
-      <c r="C49" s="5" t="n">
-        <v>30650</v>
-      </c>
-      <c r="D49" s="6" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E49" s="7" t="inlineStr">
-        <is>
-          <t>-$110.39K</t>
-        </is>
-      </c>
-      <c r="F49" s="6" t="inlineStr">
-        <is>
-          <t>+$209.75K</t>
-        </is>
-      </c>
-      <c r="G49" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H49" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>-$38.64K</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>+$226.31K</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
@@ -4632,32 +4698,36 @@
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>30767.8</v>
+        <v>30697.8</v>
       </c>
       <c r="C50" s="2" t="n">
-        <v>30760</v>
+        <v>30690</v>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E50" s="9" t="inlineStr">
-        <is>
-          <t>+$77.28K</t>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>-$60.72K</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>+$198.71K</t>
+          <t>+$215.27K</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H50" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
@@ -4666,24 +4736,24 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>30677.8</v>
+        <v>30657.8</v>
       </c>
       <c r="C51" s="5" t="n">
-        <v>30670</v>
+        <v>30650</v>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E51" s="8" t="inlineStr">
-        <is>
-          <t>+$38.64K</t>
+      <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t>-$110.39K</t>
         </is>
       </c>
       <c r="F51" s="6" t="inlineStr">
         <is>
-          <t>+$182.15K</t>
+          <t>+$209.75K</t>
         </is>
       </c>
       <c r="G51" s="6" t="inlineStr">
@@ -4693,35 +4763,35 @@
       </c>
       <c r="H51" s="6" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
-        <v>79.73999999999999</v>
+        <v>30767.8</v>
       </c>
       <c r="C52" s="2" t="n">
-        <v>130</v>
+        <v>30760</v>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E52" s="4" t="inlineStr">
-        <is>
-          <t>-$166.83K</t>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E52" s="9" t="inlineStr">
+        <is>
+          <t>+$77.28K</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>+$168.62K</t>
+          <t>+$198.71K</t>
         </is>
       </c>
       <c r="G52" s="3" t="inlineStr">
@@ -4732,76 +4802,76 @@
       <c r="H52" s="3" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="3" t="inlineStr">
+      <c r="A53" s="6" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B53" s="2" t="n">
-        <v>30607.8</v>
-      </c>
-      <c r="C53" s="2" t="n">
-        <v>30600</v>
-      </c>
-      <c r="D53" s="3" t="inlineStr">
+      <c r="B53" s="5" t="n">
+        <v>30677.8</v>
+      </c>
+      <c r="C53" s="5" t="n">
+        <v>30670</v>
+      </c>
+      <c r="D53" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E53" s="4" t="inlineStr">
-        <is>
-          <t>-$26.06K</t>
-        </is>
-      </c>
-      <c r="F53" s="3" t="inlineStr">
-        <is>
-          <t>+$161.60K</t>
-        </is>
-      </c>
-      <c r="G53" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H53" s="3" t="inlineStr"/>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>+$38.64K</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="inlineStr">
+        <is>
+          <t>+$182.15K</t>
+        </is>
+      </c>
+      <c r="G53" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H53" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>30777.8</v>
+        <v>79.73999999999999</v>
       </c>
       <c r="C54" s="2" t="n">
-        <v>30770</v>
+        <v>130</v>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E54" s="9" t="inlineStr">
-        <is>
-          <t>+$119.90K</t>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>-$166.83K</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>+$161.60K</t>
+          <t>+$168.62K</t>
         </is>
       </c>
       <c r="G54" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H54" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
@@ -4810,24 +4880,24 @@
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>30787.8</v>
+        <v>30607.8</v>
       </c>
       <c r="C55" s="2" t="n">
-        <v>30780</v>
+        <v>30600</v>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E55" s="9" t="inlineStr">
-        <is>
-          <t>+$26.06K</t>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>-$26.06K</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>+$151.18K</t>
+          <t>+$161.60K</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
@@ -4844,70 +4914,70 @@
         </is>
       </c>
       <c r="B56" s="2" t="n">
-        <v>30507.8</v>
+        <v>30777.8</v>
       </c>
       <c r="C56" s="2" t="n">
-        <v>30500</v>
+        <v>30770</v>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E56" s="4" t="inlineStr">
-        <is>
-          <t>-$127.57K</t>
+      <c r="E56" s="9" t="inlineStr">
+        <is>
+          <t>+$119.90K</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>+$143.51K</t>
+          <t>+$161.60K</t>
         </is>
       </c>
       <c r="G56" s="3" t="inlineStr">
         <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="n">
+        <v>30787.8</v>
+      </c>
+      <c r="C57" s="2" t="n">
+        <v>30780</v>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E57" s="9" t="inlineStr">
+        <is>
+          <t>+$26.06K</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>+$151.18K</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H56" s="3" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B57" s="5" t="n">
-        <v>30557.8</v>
-      </c>
-      <c r="C57" s="5" t="n">
-        <v>30550</v>
-      </c>
-      <c r="D57" s="6" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E57" s="7" t="inlineStr">
-        <is>
-          <t>-$133.39K</t>
-        </is>
-      </c>
-      <c r="F57" s="6" t="inlineStr">
-        <is>
-          <t>+$142.59K</t>
-        </is>
-      </c>
-      <c r="G57" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H57" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="H57" s="3" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
@@ -4916,24 +4986,24 @@
         </is>
       </c>
       <c r="B58" s="2" t="n">
-        <v>30857.8</v>
+        <v>30507.8</v>
       </c>
       <c r="C58" s="2" t="n">
-        <v>30850</v>
+        <v>30500</v>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E58" s="9" t="inlineStr">
-        <is>
-          <t>+$91.69K</t>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>-$127.57K</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>+$139.52K</t>
+          <t>+$143.51K</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
@@ -4944,38 +5014,42 @@
       <c r="H58" s="3" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="3" t="inlineStr">
+      <c r="A59" s="6" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B59" s="2" t="n">
-        <v>30737.8</v>
-      </c>
-      <c r="C59" s="2" t="n">
-        <v>30730</v>
-      </c>
-      <c r="D59" s="3" t="inlineStr">
+      <c r="B59" s="5" t="n">
+        <v>30557.8</v>
+      </c>
+      <c r="C59" s="5" t="n">
+        <v>30550</v>
+      </c>
+      <c r="D59" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E59" s="4" t="inlineStr">
-        <is>
-          <t>-$16.56K</t>
-        </is>
-      </c>
-      <c r="F59" s="3" t="inlineStr">
-        <is>
-          <t>+$126.95K</t>
-        </is>
-      </c>
-      <c r="G59" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H59" s="3" t="inlineStr"/>
+      <c r="E59" s="7" t="inlineStr">
+        <is>
+          <t>-$133.39K</t>
+        </is>
+      </c>
+      <c r="F59" s="6" t="inlineStr">
+        <is>
+          <t>+$142.59K</t>
+        </is>
+      </c>
+      <c r="G59" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H59" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
@@ -4984,10 +5058,10 @@
         </is>
       </c>
       <c r="B60" s="2" t="n">
-        <v>30797.8</v>
+        <v>30857.8</v>
       </c>
       <c r="C60" s="2" t="n">
-        <v>30790</v>
+        <v>30850</v>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
@@ -4996,24 +5070,20 @@
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>+$4.91K</t>
+          <t>+$91.69K</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>+$83.41K</t>
+          <t>+$139.52K</t>
         </is>
       </c>
       <c r="G60" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H60" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
@@ -5022,36 +5092,32 @@
         </is>
       </c>
       <c r="B61" s="2" t="n">
-        <v>30832.8</v>
+        <v>30737.8</v>
       </c>
       <c r="C61" s="2" t="n">
-        <v>30825</v>
+        <v>30730</v>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E61" s="9" t="inlineStr">
-        <is>
-          <t>+$9.20K</t>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>-$16.56K</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>+$46.00K</t>
+          <t>+$126.95K</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H61" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
@@ -5060,24 +5126,24 @@
         </is>
       </c>
       <c r="B62" s="2" t="n">
-        <v>30487.8</v>
+        <v>30797.8</v>
       </c>
       <c r="C62" s="2" t="n">
-        <v>30480</v>
+        <v>30790</v>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E62" s="4" t="inlineStr">
-        <is>
-          <t>-$29.44K</t>
+      <c r="E62" s="9" t="inlineStr">
+        <is>
+          <t>+$4.91K</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>+$36.80K</t>
+          <t>+$83.41K</t>
         </is>
       </c>
       <c r="G62" s="3" t="inlineStr">
@@ -5087,35 +5153,35 @@
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B63" s="2" t="n">
-        <v>83.42</v>
+        <v>30832.8</v>
       </c>
       <c r="C63" s="2" t="n">
-        <v>136</v>
+        <v>30825</v>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E63" s="4" t="inlineStr">
-        <is>
-          <t>-$19.41K</t>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E63" s="9" t="inlineStr">
+        <is>
+          <t>+$9.20K</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>+$22.46K</t>
+          <t>+$46.00K</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
@@ -5125,7 +5191,7 @@
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -5136,39 +5202,115 @@
         </is>
       </c>
       <c r="B64" s="2" t="n">
+        <v>30487.8</v>
+      </c>
+      <c r="C64" s="2" t="n">
+        <v>30480</v>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="inlineStr">
+        <is>
+          <t>-$29.44K</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>+$36.80K</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="n">
+        <v>83.42</v>
+      </c>
+      <c r="C65" s="2" t="n">
+        <v>136</v>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t>-$19.41K</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>+$22.46K</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="n">
         <v>30597.8</v>
       </c>
-      <c r="C64" s="2" t="n">
+      <c r="C66" s="2" t="n">
         <v>30590</v>
       </c>
-      <c r="D64" s="3" t="inlineStr">
+      <c r="D66" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E64" s="4" t="inlineStr">
+      <c r="E66" s="4" t="inlineStr">
         <is>
           <t>-$9.81K</t>
         </is>
       </c>
-      <c r="F64" s="3" t="inlineStr">
+      <c r="F66" s="3" t="inlineStr">
         <is>
           <t>+$9.81K</t>
         </is>
       </c>
-      <c r="G64" s="3" t="inlineStr">
+      <c r="G66" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H64" s="3" t="inlineStr">
+      <c r="H66" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H64"/>
+  <autoFilter ref="A1:H66"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>